<commit_message>
analysis of new F0AM runs, plots for Science for Solutions 2026 and 2026 Q1 UDAQ quarterly report
</commit_message>
<xml_diff>
--- a/Mechanism_info/F0AM_constraints_per_mech.xlsx
+++ b/Mechanism_info/F0AM_constraints_per_mech.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Documents\GitHub\USOS_shared\Mechanism_info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0D42A0-AE86-4976-8B1C-8D72F20B9B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D7F4F16-0162-4BEA-8C4E-EDE2B039DB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10110" yWindow="2498" windowWidth="15570" windowHeight="12165" activeTab="4" xr2:uid="{8616D58D-F8CC-4D97-8C90-BD8EB18CC822}"/>
+    <workbookView xWindow="-195" yWindow="-195" windowWidth="29190" windowHeight="15870" activeTab="4" xr2:uid="{8616D58D-F8CC-4D97-8C90-BD8EB18CC822}"/>
   </bookViews>
   <sheets>
     <sheet name="CB6r5h" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="577">
   <si>
     <t>Common_Name</t>
   </si>
@@ -1781,12 +1781,24 @@
   <si>
     <t>iPropylONO2_WAS</t>
   </si>
+  <si>
+    <t>IOLE+2*PAR</t>
+  </si>
+  <si>
+    <t>IOLE+3*PAR</t>
+  </si>
+  <si>
+    <t>ISPD</t>
+  </si>
+  <si>
+    <t>REMOVED TEMPORARILY (supposed to be NISOPNO3?)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1817,8 +1829,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1873,6 +1893,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1886,7 +1912,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1917,6 +1943,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2238,13 +2266,13 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.1328125" customWidth="1"/>
-    <col min="2" max="2" width="24.796875" customWidth="1"/>
+    <col min="2" max="2" width="24.86328125" customWidth="1"/>
     <col min="3" max="4" width="19.265625" customWidth="1"/>
     <col min="5" max="5" width="17.86328125" customWidth="1"/>
-    <col min="6" max="6" width="20.796875" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.9296875" customWidth="1"/>
-    <col min="9" max="12" width="24.796875" customWidth="1"/>
+    <col min="6" max="6" width="20.86328125" customWidth="1"/>
+    <col min="7" max="7" width="19.265625" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="12" width="24.86328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
@@ -2939,7 +2967,7 @@
   <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.19921875" customWidth="1"/>
+    <col min="1" max="1" width="29.1328125" customWidth="1"/>
     <col min="2" max="2" width="26.59765625" customWidth="1"/>
     <col min="4" max="4" width="19.59765625" customWidth="1"/>
   </cols>
@@ -4156,17 +4184,17 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="29.1328125" customWidth="1"/>
-    <col min="2" max="2" width="13.06640625" customWidth="1"/>
-    <col min="3" max="3" width="14.53125" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="14.59765625" customWidth="1"/>
     <col min="4" max="4" width="19.73046875" customWidth="1"/>
     <col min="5" max="5" width="19.73046875" style="15" customWidth="1"/>
     <col min="6" max="6" width="30.3984375" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="13.73046875" customWidth="1"/>
-    <col min="8" max="8" width="17.796875" customWidth="1"/>
-    <col min="9" max="9" width="12.19921875" customWidth="1"/>
-    <col min="10" max="10" width="30.53125" customWidth="1"/>
+    <col min="8" max="8" width="17.86328125" customWidth="1"/>
+    <col min="9" max="9" width="12.1328125" customWidth="1"/>
+    <col min="10" max="10" width="30.59765625" customWidth="1"/>
     <col min="11" max="11" width="21.1328125" customWidth="1"/>
-    <col min="12" max="13" width="9.06640625" customWidth="1"/>
+    <col min="12" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="14.265625" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="16.73046875" customWidth="1"/>
   </cols>
@@ -4542,13 +4570,13 @@
       <c r="A12" t="s">
         <v>265</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="26" t="s">
         <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>267</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="26" t="s">
         <v>157</v>
       </c>
       <c r="E12" s="19" t="s">
@@ -4560,10 +4588,10 @@
       <c r="H12" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="I12" s="24" t="s">
+      <c r="I12" s="26" t="s">
         <v>280</v>
       </c>
-      <c r="J12" s="24" t="s">
+      <c r="J12" s="26" t="s">
         <v>124</v>
       </c>
       <c r="K12" t="s">
@@ -4580,11 +4608,11 @@
       <c r="A13" t="s">
         <v>264</v>
       </c>
-      <c r="B13" s="24"/>
+      <c r="B13" s="26"/>
       <c r="C13" t="s">
         <v>266</v>
       </c>
-      <c r="D13" s="24"/>
+      <c r="D13" s="26"/>
       <c r="E13" s="16" t="s">
         <v>481</v>
       </c>
@@ -4594,8 +4622,8 @@
       <c r="H13" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
       <c r="K13" t="s">
         <v>392</v>
       </c>
@@ -4610,19 +4638,19 @@
       <c r="A14" s="20" t="s">
         <v>482</v>
       </c>
-      <c r="B14" s="24"/>
+      <c r="B14" s="26"/>
       <c r="C14" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="D14" s="24"/>
+      <c r="D14" s="26"/>
       <c r="E14" s="16" t="s">
         <v>483</v>
       </c>
       <c r="H14" s="14" t="s">
         <v>528</v>
       </c>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
       <c r="O14" s="15" t="s">
         <v>531</v>
       </c>
@@ -6230,13 +6258,13 @@
       <c r="A72" t="s">
         <v>552</v>
       </c>
-      <c r="B72" s="24" t="s">
+      <c r="B72" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="C72" s="24" t="s">
+      <c r="C72" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="D72" s="24" t="s">
+      <c r="D72" s="26" t="s">
         <v>185</v>
       </c>
       <c r="E72" s="4" t="s">
@@ -6259,9 +6287,9 @@
       <c r="A73" s="21" t="s">
         <v>551</v>
       </c>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="26"/>
       <c r="E73" s="4" t="s">
         <v>554</v>
       </c>
@@ -6843,8 +6871,11 @@
   <dimension ref="A1:O99"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.46484375" style="21" customWidth="1"/>
-    <col min="2" max="16384" width="10.59765625" style="21"/>
+    <col min="1" max="1" width="20.3984375" style="21" customWidth="1"/>
+    <col min="2" max="7" width="0" style="21" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="26.86328125" style="21" customWidth="1"/>
+    <col min="9" max="14" width="0" style="21" hidden="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.59765625" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.45">
@@ -7096,13 +7127,13 @@
       <c r="A12" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="26" t="s">
         <v>87</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>267</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="26" t="s">
         <v>157</v>
       </c>
       <c r="E12" s="19" t="s">
@@ -7114,8 +7145,8 @@
       <c r="H12" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24" t="s">
+      <c r="I12" s="26"/>
+      <c r="J12" s="26" t="s">
         <v>124</v>
       </c>
       <c r="K12" s="21" t="s">
@@ -7129,24 +7160,21 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B13" s="24"/>
-      <c r="C13" s="21" t="s">
-        <v>266</v>
-      </c>
-      <c r="D13" s="24"/>
+      <c r="B13" s="26"/>
+      <c r="D13" s="26"/>
       <c r="E13" s="22"/>
       <c r="H13" s="22"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A14" s="20"/>
-      <c r="B14" s="24"/>
-      <c r="D14" s="24"/>
+      <c r="B14" s="26"/>
+      <c r="D14" s="26"/>
       <c r="E14" s="22"/>
       <c r="H14" s="22"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A16" s="21" t="s">
@@ -7427,7 +7455,7 @@
         <v>275</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>422</v>
+        <v>575</v>
       </c>
       <c r="C24" s="21" t="s">
         <v>277</v>
@@ -7545,8 +7573,8 @@
       <c r="A31" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>104</v>
+      <c r="B31" s="25" t="s">
+        <v>151</v>
       </c>
       <c r="C31" s="21" t="s">
         <v>205</v>
@@ -7574,8 +7602,8 @@
       <c r="A32" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="B32" s="21" t="s">
-        <v>104</v>
+      <c r="B32" s="25" t="s">
+        <v>151</v>
       </c>
       <c r="C32" s="21" t="s">
         <v>205</v>
@@ -7603,8 +7631,8 @@
       <c r="A33" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="B33" s="21" t="s">
-        <v>106</v>
+      <c r="B33" s="25" t="s">
+        <v>104</v>
       </c>
       <c r="C33" s="21" t="s">
         <v>196</v>
@@ -7632,8 +7660,8 @@
       <c r="A34" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="B34" s="21" t="s">
-        <v>106</v>
+      <c r="B34" s="25" t="s">
+        <v>104</v>
       </c>
       <c r="C34" s="21" t="s">
         <v>196</v>
@@ -7671,8 +7699,8 @@
       <c r="A38" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="B38" s="21" t="s">
-        <v>107</v>
+      <c r="B38" s="25" t="s">
+        <v>106</v>
       </c>
       <c r="C38" s="21" t="s">
         <v>196</v>
@@ -7717,8 +7745,8 @@
       <c r="A46" s="21" t="s">
         <v>304</v>
       </c>
-      <c r="B46" s="21" t="s">
-        <v>109</v>
+      <c r="B46" s="25" t="s">
+        <v>108</v>
       </c>
       <c r="C46" s="21" t="s">
         <v>210</v>
@@ -7746,8 +7774,8 @@
       <c r="A47" s="21" t="s">
         <v>305</v>
       </c>
-      <c r="B47" s="21" t="s">
-        <v>110</v>
+      <c r="B47" s="25" t="s">
+        <v>109</v>
       </c>
       <c r="C47" s="21" t="s">
         <v>210</v>
@@ -7775,8 +7803,8 @@
       <c r="A48" s="21" t="s">
         <v>306</v>
       </c>
-      <c r="B48" s="21" t="s">
-        <v>111</v>
+      <c r="B48" s="25" t="s">
+        <v>110</v>
       </c>
       <c r="C48" s="21" t="s">
         <v>210</v>
@@ -7904,7 +7932,7 @@
       <c r="A58" s="21" t="s">
         <v>371</v>
       </c>
-      <c r="B58" s="21" t="s">
+      <c r="B58" s="25" t="s">
         <v>333</v>
       </c>
       <c r="C58" s="21" t="s">
@@ -7933,8 +7961,8 @@
       <c r="A59" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="B59" s="21" t="s">
-        <v>105</v>
+      <c r="B59" s="25" t="s">
+        <v>573</v>
       </c>
       <c r="C59" s="21" t="s">
         <v>208</v>
@@ -7962,8 +7990,8 @@
       <c r="A60" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="B60" s="21" t="s">
-        <v>105</v>
+      <c r="B60" s="25" t="s">
+        <v>573</v>
       </c>
       <c r="C60" s="21" t="s">
         <v>208</v>
@@ -7991,7 +8019,7 @@
       <c r="A61" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="B61" s="21" t="s">
+      <c r="B61" s="25" t="s">
         <v>335</v>
       </c>
       <c r="C61" s="21" t="s">
@@ -8020,8 +8048,8 @@
       <c r="A62" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="B62" s="21" t="s">
-        <v>336</v>
+      <c r="B62" s="25" t="s">
+        <v>574</v>
       </c>
       <c r="C62" s="21" t="s">
         <v>208</v>
@@ -8049,8 +8077,8 @@
       <c r="A63" s="21" t="s">
         <v>300</v>
       </c>
-      <c r="B63" s="21" t="s">
-        <v>336</v>
+      <c r="B63" s="25" t="s">
+        <v>574</v>
       </c>
       <c r="C63" s="21" t="s">
         <v>208</v>
@@ -8082,7 +8110,7 @@
       <c r="A65" s="21" t="s">
         <v>315</v>
       </c>
-      <c r="B65" s="21" t="s">
+      <c r="B65" s="25" t="s">
         <v>338</v>
       </c>
       <c r="C65" s="21" t="s">
@@ -8115,8 +8143,8 @@
       <c r="A67" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="B67" s="21" t="s">
-        <v>107</v>
+      <c r="B67" s="25" t="s">
+        <v>106</v>
       </c>
       <c r="C67" s="21" t="s">
         <v>196</v>
@@ -8159,7 +8187,7 @@
       <c r="A71" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="B71" s="21" t="s">
+      <c r="B71" s="25" t="s">
         <v>339</v>
       </c>
       <c r="C71" s="21" t="s">
@@ -8188,13 +8216,13 @@
       <c r="A72" s="21" t="s">
         <v>552</v>
       </c>
-      <c r="B72" s="24" t="s">
+      <c r="B72" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="C72" s="24" t="s">
+      <c r="C72" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="D72" s="24" t="s">
+      <c r="D72" s="26" t="s">
         <v>185</v>
       </c>
       <c r="E72" s="4" t="s">
@@ -8217,9 +8245,9 @@
       <c r="A73" s="21" t="s">
         <v>551</v>
       </c>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="26"/>
       <c r="E73" s="4" t="s">
         <v>554</v>
       </c>
@@ -8303,8 +8331,12 @@
       <c r="B87" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="C87" s="3"/>
-      <c r="D87" s="3"/>
+      <c r="C87" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>271</v>
+      </c>
       <c r="E87" s="4" t="s">
         <v>524</v>
       </c>
@@ -8316,46 +8348,53 @@
       </c>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B88" s="3"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="3"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
       <c r="E88" s="4"/>
       <c r="H88" s="9"/>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B89" s="3"/>
-      <c r="C89" s="3"/>
-      <c r="E89" s="3"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
       <c r="H89" s="8"/>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B90" s="3"/>
-      <c r="C90" s="3"/>
-      <c r="E90" s="3"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
       <c r="H90" s="8"/>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B91" s="3"/>
-      <c r="C91" s="3"/>
-      <c r="E91" s="3"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
       <c r="H91" s="8"/>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B92" s="3"/>
-      <c r="C92" s="3"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
       <c r="H92" s="8"/>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="B93" s="3"/>
-      <c r="C93" s="3"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
       <c r="H93" s="8"/>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A94" s="21" t="s">
         <v>419</v>
       </c>
-      <c r="B94" s="13" t="s">
-        <v>475</v>
+      <c r="B94" s="3" t="s">
+        <v>271</v>
       </c>
       <c r="C94" s="21" t="s">
         <v>421</v>
@@ -8380,6 +8419,9 @@
       <c r="A96" s="21" t="s">
         <v>541</v>
       </c>
+      <c r="B96" s="6" t="s">
+        <v>422</v>
+      </c>
       <c r="C96" s="21" t="s">
         <v>568</v>
       </c>
@@ -8400,6 +8442,9 @@
       <c r="A97" s="21" t="s">
         <v>545</v>
       </c>
+      <c r="B97" s="21" t="s">
+        <v>575</v>
+      </c>
       <c r="C97" s="21" t="s">
         <v>545</v>
       </c>
@@ -8426,6 +8471,9 @@
       <c r="A98" s="21" t="s">
         <v>548</v>
       </c>
+      <c r="B98" s="21" t="s">
+        <v>575</v>
+      </c>
       <c r="C98" s="21" t="s">
         <v>548</v>
       </c>
@@ -8443,8 +8491,8 @@
       </c>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A99" s="21" t="s">
-        <v>556</v>
+      <c r="A99" s="24" t="s">
+        <v>576</v>
       </c>
       <c r="D99" s="21" t="s">
         <v>569</v>
@@ -8459,7 +8507,7 @@
         <v>571</v>
       </c>
       <c r="O99" s="21" t="s">
-        <v>533</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>

</xml_diff>